<commit_message>
Update da Base de Dados
Completando a coluna de "Ambientes"
</commit_message>
<xml_diff>
--- a/dados_projeto.xlsx
+++ b/dados_projeto.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JR\Desktop\Projeto_Enxoval\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9050f00462f35375/Desktop/PYTHON/Projeto_Enxoval/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61F9F760-CB75-4513-AE38-A32BB50E1E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{61F9F760-CB75-4513-AE38-A32BB50E1E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DAF5E58-8A92-4FAF-AC12-98532E19C70D}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="219">
   <si>
     <t>Ambiente</t>
   </si>
@@ -529,15 +529,9 @@
     <t>Cuba</t>
   </si>
   <si>
-    <t>Cortina p/ box</t>
-  </si>
-  <si>
     <t>Tapete Box</t>
   </si>
   <si>
-    <t>Toalha pés</t>
-  </si>
-  <si>
     <t>Cama Box/ Colchão</t>
   </si>
   <si>
@@ -671,6 +665,18 @@
   </si>
   <si>
     <t>Cozinha</t>
+  </si>
+  <si>
+    <t>Sala</t>
+  </si>
+  <si>
+    <t>Quarto</t>
+  </si>
+  <si>
+    <t>Lavanderia</t>
+  </si>
+  <si>
+    <t>Banheiro</t>
   </si>
 </sst>
 </file>
@@ -1010,8 +1016,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G212"/>
+  <dimension ref="A1:G210"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -1038,7 +1048,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -1058,7 +1068,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -1078,7 +1088,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
@@ -1098,7 +1108,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
@@ -1117,6 +1127,9 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>214</v>
+      </c>
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -1134,6 +1147,9 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>214</v>
+      </c>
       <c r="B7" t="s">
         <v>13</v>
       </c>
@@ -1151,6 +1167,9 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>214</v>
+      </c>
       <c r="B8" t="s">
         <v>14</v>
       </c>
@@ -1168,6 +1187,9 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>214</v>
+      </c>
       <c r="B9" t="s">
         <v>15</v>
       </c>
@@ -1185,6 +1207,9 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>214</v>
+      </c>
       <c r="B10" t="s">
         <v>16</v>
       </c>
@@ -1202,6 +1227,9 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>214</v>
+      </c>
       <c r="B11" t="s">
         <v>17</v>
       </c>
@@ -1219,6 +1247,9 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>214</v>
+      </c>
       <c r="B12" t="s">
         <v>18</v>
       </c>
@@ -1236,6 +1267,9 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>214</v>
+      </c>
       <c r="B13" t="s">
         <v>19</v>
       </c>
@@ -1253,6 +1287,9 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>214</v>
+      </c>
       <c r="B14" t="s">
         <v>20</v>
       </c>
@@ -1270,6 +1307,9 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>214</v>
+      </c>
       <c r="B15" t="s">
         <v>21</v>
       </c>
@@ -1287,6 +1327,9 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>214</v>
+      </c>
       <c r="B16" t="s">
         <v>22</v>
       </c>
@@ -1303,7 +1346,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>214</v>
+      </c>
       <c r="B17" t="s">
         <v>23</v>
       </c>
@@ -1320,7 +1366,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>214</v>
+      </c>
       <c r="B18" t="s">
         <v>24</v>
       </c>
@@ -1337,7 +1386,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>214</v>
+      </c>
       <c r="B19" t="s">
         <v>25</v>
       </c>
@@ -1354,7 +1406,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>214</v>
+      </c>
       <c r="B20" t="s">
         <v>26</v>
       </c>
@@ -1371,7 +1426,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>214</v>
+      </c>
       <c r="B21" t="s">
         <v>27</v>
       </c>
@@ -1388,7 +1446,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>215</v>
+      </c>
       <c r="B22" t="s">
         <v>28</v>
       </c>
@@ -1405,7 +1466,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>215</v>
+      </c>
       <c r="B23" t="s">
         <v>29</v>
       </c>
@@ -1422,7 +1486,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>215</v>
+      </c>
       <c r="B24" t="s">
         <v>30</v>
       </c>
@@ -1439,7 +1506,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>215</v>
+      </c>
       <c r="B25" t="s">
         <v>31</v>
       </c>
@@ -1456,7 +1526,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>215</v>
+      </c>
       <c r="B26" t="s">
         <v>32</v>
       </c>
@@ -1473,7 +1546,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>215</v>
+      </c>
       <c r="B27" t="s">
         <v>33</v>
       </c>
@@ -1490,7 +1566,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>215</v>
+      </c>
       <c r="B28" t="s">
         <v>34</v>
       </c>
@@ -1507,7 +1586,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>216</v>
+      </c>
       <c r="B29" t="s">
         <v>35</v>
       </c>
@@ -1524,7 +1606,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>216</v>
+      </c>
       <c r="B30" t="s">
         <v>36</v>
       </c>
@@ -1541,7 +1626,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>214</v>
+      </c>
       <c r="B31" t="s">
         <v>37</v>
       </c>
@@ -1558,7 +1646,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>214</v>
+      </c>
       <c r="B32" t="s">
         <v>38</v>
       </c>
@@ -1575,7 +1666,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>214</v>
+      </c>
       <c r="B33" t="s">
         <v>39</v>
       </c>
@@ -1592,7 +1686,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>214</v>
+      </c>
       <c r="B34" t="s">
         <v>40</v>
       </c>
@@ -1609,7 +1706,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>214</v>
+      </c>
       <c r="B35" t="s">
         <v>41</v>
       </c>
@@ -1626,7 +1726,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>214</v>
+      </c>
       <c r="B36" t="s">
         <v>42</v>
       </c>
@@ -1643,7 +1746,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>214</v>
+      </c>
       <c r="B37" t="s">
         <v>43</v>
       </c>
@@ -1660,7 +1766,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>214</v>
+      </c>
       <c r="B38" t="s">
         <v>44</v>
       </c>
@@ -1677,7 +1786,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>214</v>
+      </c>
       <c r="B39" t="s">
         <v>45</v>
       </c>
@@ -1694,7 +1806,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>214</v>
+      </c>
       <c r="B40" t="s">
         <v>46</v>
       </c>
@@ -1711,7 +1826,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>214</v>
+      </c>
       <c r="B41" t="s">
         <v>47</v>
       </c>
@@ -1728,7 +1846,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>214</v>
+      </c>
       <c r="B42" t="s">
         <v>48</v>
       </c>
@@ -1745,7 +1866,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>214</v>
+      </c>
       <c r="B43" t="s">
         <v>49</v>
       </c>
@@ -1762,7 +1886,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>214</v>
+      </c>
       <c r="B44" t="s">
         <v>50</v>
       </c>
@@ -1779,7 +1906,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>214</v>
+      </c>
       <c r="B45" t="s">
         <v>51</v>
       </c>
@@ -1796,7 +1926,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>214</v>
+      </c>
       <c r="B46" t="s">
         <v>52</v>
       </c>
@@ -1813,7 +1946,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>214</v>
+      </c>
       <c r="B47" t="s">
         <v>53</v>
       </c>
@@ -1830,7 +1966,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>214</v>
+      </c>
       <c r="B48" t="s">
         <v>54</v>
       </c>
@@ -1847,7 +1986,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>217</v>
+      </c>
       <c r="B49" t="s">
         <v>55</v>
       </c>
@@ -1864,7 +2006,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>214</v>
+      </c>
       <c r="B50" t="s">
         <v>56</v>
       </c>
@@ -1881,7 +2026,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>214</v>
+      </c>
       <c r="B51" t="s">
         <v>57</v>
       </c>
@@ -1898,7 +2046,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>214</v>
+      </c>
       <c r="B52" t="s">
         <v>58</v>
       </c>
@@ -1915,7 +2066,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>214</v>
+      </c>
       <c r="B53" t="s">
         <v>59</v>
       </c>
@@ -1932,7 +2086,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>214</v>
+      </c>
       <c r="B54" t="s">
         <v>60</v>
       </c>
@@ -1949,7 +2106,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>214</v>
+      </c>
       <c r="B55" t="s">
         <v>61</v>
       </c>
@@ -1966,7 +2126,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>214</v>
+      </c>
       <c r="B56" t="s">
         <v>62</v>
       </c>
@@ -1983,7 +2146,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>214</v>
+      </c>
       <c r="B57" t="s">
         <v>63</v>
       </c>
@@ -2000,7 +2166,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>214</v>
+      </c>
       <c r="B58" t="s">
         <v>64</v>
       </c>
@@ -2017,7 +2186,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>214</v>
+      </c>
       <c r="B59" t="s">
         <v>65</v>
       </c>
@@ -2034,7 +2206,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>214</v>
+      </c>
       <c r="B60" t="s">
         <v>66</v>
       </c>
@@ -2051,7 +2226,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>214</v>
+      </c>
       <c r="B61" t="s">
         <v>67</v>
       </c>
@@ -2068,7 +2246,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>214</v>
+      </c>
       <c r="B62" t="s">
         <v>68</v>
       </c>
@@ -2085,7 +2266,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>214</v>
+      </c>
       <c r="B63" t="s">
         <v>69</v>
       </c>
@@ -2102,7 +2286,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>214</v>
+      </c>
       <c r="B64" t="s">
         <v>70</v>
       </c>
@@ -2119,7 +2306,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>214</v>
+      </c>
       <c r="B65" t="s">
         <v>71</v>
       </c>
@@ -2136,7 +2326,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>214</v>
+      </c>
       <c r="B66" t="s">
         <v>72</v>
       </c>
@@ -2153,7 +2346,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>214</v>
+      </c>
       <c r="B67" t="s">
         <v>73</v>
       </c>
@@ -2170,7 +2366,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>214</v>
+      </c>
       <c r="B68" t="s">
         <v>74</v>
       </c>
@@ -2187,7 +2386,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>214</v>
+      </c>
       <c r="B69" t="s">
         <v>75</v>
       </c>
@@ -2204,7 +2406,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>214</v>
+      </c>
       <c r="B70" t="s">
         <v>76</v>
       </c>
@@ -2221,7 +2426,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>214</v>
+      </c>
       <c r="B71" t="s">
         <v>77</v>
       </c>
@@ -2238,7 +2446,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>214</v>
+      </c>
       <c r="B72" t="s">
         <v>78</v>
       </c>
@@ -2255,7 +2466,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>214</v>
+      </c>
       <c r="B73" t="s">
         <v>79</v>
       </c>
@@ -2272,7 +2486,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>214</v>
+      </c>
       <c r="B74" t="s">
         <v>80</v>
       </c>
@@ -2289,7 +2506,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>214</v>
+      </c>
       <c r="B75" t="s">
         <v>81</v>
       </c>
@@ -2306,7 +2526,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>214</v>
+      </c>
       <c r="B76" t="s">
         <v>82</v>
       </c>
@@ -2323,7 +2546,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>214</v>
+      </c>
       <c r="B77" t="s">
         <v>83</v>
       </c>
@@ -2340,7 +2566,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>214</v>
+      </c>
       <c r="B78" t="s">
         <v>84</v>
       </c>
@@ -2357,7 +2586,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>214</v>
+      </c>
       <c r="B79" t="s">
         <v>85</v>
       </c>
@@ -2374,7 +2606,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>214</v>
+      </c>
       <c r="B80" t="s">
         <v>86</v>
       </c>
@@ -2391,7 +2626,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>214</v>
+      </c>
       <c r="B81" t="s">
         <v>87</v>
       </c>
@@ -2408,7 +2646,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>214</v>
+      </c>
       <c r="B82" t="s">
         <v>88</v>
       </c>
@@ -2425,7 +2666,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>214</v>
+      </c>
       <c r="B83" t="s">
         <v>89</v>
       </c>
@@ -2442,7 +2686,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>214</v>
+      </c>
       <c r="B84" t="s">
         <v>90</v>
       </c>
@@ -2459,7 +2706,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>214</v>
+      </c>
       <c r="B85" t="s">
         <v>91</v>
       </c>
@@ -2476,7 +2726,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>214</v>
+      </c>
       <c r="B86" t="s">
         <v>92</v>
       </c>
@@ -2493,7 +2746,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>214</v>
+      </c>
       <c r="B87" t="s">
         <v>93</v>
       </c>
@@ -2510,7 +2766,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>214</v>
+      </c>
       <c r="B88" t="s">
         <v>94</v>
       </c>
@@ -2527,7 +2786,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>214</v>
+      </c>
       <c r="B89" t="s">
         <v>95</v>
       </c>
@@ -2544,7 +2806,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>214</v>
+      </c>
       <c r="B90" t="s">
         <v>96</v>
       </c>
@@ -2561,7 +2826,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>214</v>
+      </c>
       <c r="B91" t="s">
         <v>97</v>
       </c>
@@ -2578,7 +2846,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>214</v>
+      </c>
       <c r="B92" t="s">
         <v>98</v>
       </c>
@@ -2595,7 +2866,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>214</v>
+      </c>
       <c r="B93" t="s">
         <v>99</v>
       </c>
@@ -2612,7 +2886,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>214</v>
+      </c>
       <c r="B94" t="s">
         <v>100</v>
       </c>
@@ -2629,7 +2906,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>214</v>
+      </c>
       <c r="B95" t="s">
         <v>101</v>
       </c>
@@ -2646,7 +2926,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>214</v>
+      </c>
       <c r="B96" t="s">
         <v>102</v>
       </c>
@@ -2663,7 +2946,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>214</v>
+      </c>
       <c r="B97" t="s">
         <v>103</v>
       </c>
@@ -2680,7 +2966,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>214</v>
+      </c>
       <c r="B98" t="s">
         <v>104</v>
       </c>
@@ -2697,7 +2986,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>214</v>
+      </c>
       <c r="B99" t="s">
         <v>105</v>
       </c>
@@ -2714,7 +3006,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>214</v>
+      </c>
       <c r="B100" t="s">
         <v>106</v>
       </c>
@@ -2731,7 +3026,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>214</v>
+      </c>
       <c r="B101" t="s">
         <v>107</v>
       </c>
@@ -2748,7 +3046,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="102" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>214</v>
+      </c>
       <c r="B102" t="s">
         <v>108</v>
       </c>
@@ -2765,7 +3066,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="103" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>214</v>
+      </c>
       <c r="B103" t="s">
         <v>109</v>
       </c>
@@ -2782,7 +3086,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="104" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>214</v>
+      </c>
       <c r="B104" t="s">
         <v>110</v>
       </c>
@@ -2799,7 +3106,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="105" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>214</v>
+      </c>
       <c r="B105" t="s">
         <v>111</v>
       </c>
@@ -2816,7 +3126,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="106" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>214</v>
+      </c>
       <c r="B106" t="s">
         <v>112</v>
       </c>
@@ -2833,7 +3146,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="107" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>214</v>
+      </c>
       <c r="B107" t="s">
         <v>113</v>
       </c>
@@ -2850,7 +3166,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="108" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>214</v>
+      </c>
       <c r="B108" t="s">
         <v>114</v>
       </c>
@@ -2867,7 +3186,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="109" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>214</v>
+      </c>
       <c r="B109" t="s">
         <v>115</v>
       </c>
@@ -2884,7 +3206,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="110" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>214</v>
+      </c>
       <c r="B110" t="s">
         <v>116</v>
       </c>
@@ -2901,7 +3226,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="111" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>214</v>
+      </c>
       <c r="B111" t="s">
         <v>117</v>
       </c>
@@ -2918,7 +3246,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="112" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>214</v>
+      </c>
       <c r="B112" t="s">
         <v>118</v>
       </c>
@@ -2935,7 +3266,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="113" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>214</v>
+      </c>
       <c r="B113" t="s">
         <v>119</v>
       </c>
@@ -2952,7 +3286,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="114" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>214</v>
+      </c>
       <c r="B114" t="s">
         <v>120</v>
       </c>
@@ -2969,7 +3306,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="115" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>214</v>
+      </c>
       <c r="B115" t="s">
         <v>121</v>
       </c>
@@ -2986,7 +3326,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="116" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>214</v>
+      </c>
       <c r="B116" t="s">
         <v>122</v>
       </c>
@@ -3003,7 +3346,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="117" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>214</v>
+      </c>
       <c r="B117" t="s">
         <v>123</v>
       </c>
@@ -3020,7 +3366,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="118" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>214</v>
+      </c>
       <c r="B118" t="s">
         <v>124</v>
       </c>
@@ -3037,7 +3386,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="119" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>214</v>
+      </c>
       <c r="B119" t="s">
         <v>125</v>
       </c>
@@ -3054,7 +3406,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="120" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>214</v>
+      </c>
       <c r="B120" t="s">
         <v>126</v>
       </c>
@@ -3071,7 +3426,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="121" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>214</v>
+      </c>
       <c r="B121" t="s">
         <v>127</v>
       </c>
@@ -3088,7 +3446,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="122" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>214</v>
+      </c>
       <c r="B122" t="s">
         <v>128</v>
       </c>
@@ -3105,7 +3466,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="123" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>214</v>
+      </c>
       <c r="B123" t="s">
         <v>129</v>
       </c>
@@ -3122,7 +3486,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="124" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>214</v>
+      </c>
       <c r="B124" t="s">
         <v>130</v>
       </c>
@@ -3139,7 +3506,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="125" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>214</v>
+      </c>
       <c r="B125" t="s">
         <v>131</v>
       </c>
@@ -3156,7 +3526,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="126" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>214</v>
+      </c>
       <c r="B126" t="s">
         <v>132</v>
       </c>
@@ -3173,7 +3546,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="127" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>217</v>
+      </c>
       <c r="B127" t="s">
         <v>133</v>
       </c>
@@ -3190,7 +3566,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="128" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>217</v>
+      </c>
       <c r="B128" t="s">
         <v>134</v>
       </c>
@@ -3207,7 +3586,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="129" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>217</v>
+      </c>
       <c r="B129" t="s">
         <v>135</v>
       </c>
@@ -3224,7 +3606,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="130" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>217</v>
+      </c>
       <c r="B130" t="s">
         <v>136</v>
       </c>
@@ -3241,7 +3626,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="131" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>217</v>
+      </c>
       <c r="B131" t="s">
         <v>137</v>
       </c>
@@ -3258,7 +3646,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="132" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>217</v>
+      </c>
       <c r="B132" t="s">
         <v>138</v>
       </c>
@@ -3275,7 +3666,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="133" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>217</v>
+      </c>
       <c r="B133" t="s">
         <v>139</v>
       </c>
@@ -3292,7 +3686,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="134" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>217</v>
+      </c>
       <c r="B134" t="s">
         <v>140</v>
       </c>
@@ -3309,7 +3706,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="135" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>217</v>
+      </c>
       <c r="B135" t="s">
         <v>141</v>
       </c>
@@ -3326,7 +3726,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="136" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>217</v>
+      </c>
       <c r="B136" t="s">
         <v>142</v>
       </c>
@@ -3343,7 +3746,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="137" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>217</v>
+      </c>
       <c r="B137" t="s">
         <v>143</v>
       </c>
@@ -3360,7 +3766,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="138" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>217</v>
+      </c>
       <c r="B138" t="s">
         <v>55</v>
       </c>
@@ -3377,7 +3786,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="139" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>217</v>
+      </c>
       <c r="B139" t="s">
         <v>144</v>
       </c>
@@ -3394,7 +3806,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="140" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>217</v>
+      </c>
       <c r="B140" t="s">
         <v>145</v>
       </c>
@@ -3411,7 +3826,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="141" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>217</v>
+      </c>
       <c r="B141" t="s">
         <v>146</v>
       </c>
@@ -3428,7 +3846,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="142" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>217</v>
+      </c>
       <c r="B142" t="s">
         <v>147</v>
       </c>
@@ -3445,7 +3866,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="143" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>217</v>
+      </c>
       <c r="B143" t="s">
         <v>148</v>
       </c>
@@ -3462,7 +3886,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="144" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>217</v>
+      </c>
       <c r="B144" t="s">
         <v>149</v>
       </c>
@@ -3479,7 +3906,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="145" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>217</v>
+      </c>
       <c r="B145" t="s">
         <v>150</v>
       </c>
@@ -3496,7 +3926,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="146" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>217</v>
+      </c>
       <c r="B146" t="s">
         <v>151</v>
       </c>
@@ -3513,7 +3946,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="147" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>218</v>
+      </c>
       <c r="B147" t="s">
         <v>152</v>
       </c>
@@ -3530,7 +3966,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="148" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>218</v>
+      </c>
       <c r="B148" t="s">
         <v>153</v>
       </c>
@@ -3547,7 +3986,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="149" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>218</v>
+      </c>
       <c r="B149" t="s">
         <v>154</v>
       </c>
@@ -3564,7 +4006,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="150" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>218</v>
+      </c>
       <c r="B150" t="s">
         <v>155</v>
       </c>
@@ -3581,7 +4026,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="151" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>218</v>
+      </c>
       <c r="B151" t="s">
         <v>156</v>
       </c>
@@ -3598,7 +4046,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="152" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>218</v>
+      </c>
       <c r="B152" t="s">
         <v>157</v>
       </c>
@@ -3615,7 +4066,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="153" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>218</v>
+      </c>
       <c r="B153" t="s">
         <v>158</v>
       </c>
@@ -3632,7 +4086,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="154" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>218</v>
+      </c>
       <c r="B154" t="s">
         <v>159</v>
       </c>
@@ -3649,7 +4106,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="155" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>218</v>
+      </c>
       <c r="B155" t="s">
         <v>160</v>
       </c>
@@ -3666,7 +4126,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="156" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>218</v>
+      </c>
       <c r="B156" t="s">
         <v>161</v>
       </c>
@@ -3683,7 +4146,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="157" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>218</v>
+      </c>
       <c r="B157" t="s">
         <v>162</v>
       </c>
@@ -3700,7 +4166,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="158" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>218</v>
+      </c>
       <c r="B158" t="s">
         <v>163</v>
       </c>
@@ -3717,7 +4186,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="159" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>218</v>
+      </c>
       <c r="B159" t="s">
         <v>164</v>
       </c>
@@ -3734,7 +4206,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="160" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>218</v>
+      </c>
       <c r="B160" t="s">
         <v>165</v>
       </c>
@@ -3751,7 +4226,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="161" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>218</v>
+      </c>
       <c r="B161" t="s">
         <v>166</v>
       </c>
@@ -3768,7 +4246,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="162" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>218</v>
+      </c>
       <c r="B162" t="s">
         <v>167</v>
       </c>
@@ -3785,7 +4266,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="163" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>218</v>
+      </c>
       <c r="B163" t="s">
         <v>168</v>
       </c>
@@ -3802,7 +4286,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="164" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>218</v>
+      </c>
       <c r="B164" t="s">
         <v>169</v>
       </c>
@@ -3819,7 +4306,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="165" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>216</v>
+      </c>
       <c r="B165" t="s">
         <v>170</v>
       </c>
@@ -3836,7 +4326,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="166" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>216</v>
+      </c>
       <c r="B166" t="s">
         <v>171</v>
       </c>
@@ -3853,44 +4346,53 @@
         <v>8</v>
       </c>
     </row>
-    <row r="167" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>216</v>
+      </c>
       <c r="B167" t="s">
+        <v>154</v>
+      </c>
+      <c r="C167">
+        <v>0</v>
+      </c>
+      <c r="D167">
+        <v>0</v>
+      </c>
+      <c r="E167">
+        <v>0</v>
+      </c>
+      <c r="F167" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>216</v>
+      </c>
+      <c r="B168" t="s">
         <v>172</v>
       </c>
-      <c r="C167">
-        <v>0</v>
-      </c>
-      <c r="D167">
-        <v>0</v>
-      </c>
-      <c r="E167">
-        <v>0</v>
-      </c>
-      <c r="F167" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="168" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B168" t="s">
+      <c r="C168">
+        <v>0</v>
+      </c>
+      <c r="D168">
+        <v>0</v>
+      </c>
+      <c r="E168">
+        <v>0</v>
+      </c>
+      <c r="F168" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>216</v>
+      </c>
+      <c r="B169" t="s">
         <v>173</v>
       </c>
-      <c r="C168">
-        <v>0</v>
-      </c>
-      <c r="D168">
-        <v>0</v>
-      </c>
-      <c r="E168">
-        <v>0</v>
-      </c>
-      <c r="F168" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="169" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B169" t="s">
-        <v>154</v>
-      </c>
       <c r="C169">
         <v>0</v>
       </c>
@@ -3904,7 +4406,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="170" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>216</v>
+      </c>
       <c r="B170" t="s">
         <v>174</v>
       </c>
@@ -3921,7 +4426,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="171" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>216</v>
+      </c>
       <c r="B171" t="s">
         <v>175</v>
       </c>
@@ -3938,7 +4446,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="172" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>216</v>
+      </c>
       <c r="B172" t="s">
         <v>176</v>
       </c>
@@ -3955,7 +4466,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="173" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>216</v>
+      </c>
       <c r="B173" t="s">
         <v>177</v>
       </c>
@@ -3972,7 +4486,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="174" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>216</v>
+      </c>
       <c r="B174" t="s">
         <v>178</v>
       </c>
@@ -3989,7 +4506,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="175" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>216</v>
+      </c>
       <c r="B175" t="s">
         <v>179</v>
       </c>
@@ -4006,7 +4526,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="176" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>216</v>
+      </c>
       <c r="B176" t="s">
         <v>180</v>
       </c>
@@ -4023,7 +4546,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="177" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>216</v>
+      </c>
       <c r="B177" t="s">
         <v>181</v>
       </c>
@@ -4040,7 +4566,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="178" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>216</v>
+      </c>
       <c r="B178" t="s">
         <v>182</v>
       </c>
@@ -4057,7 +4586,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="179" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>216</v>
+      </c>
       <c r="B179" t="s">
         <v>183</v>
       </c>
@@ -4074,7 +4606,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="180" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>216</v>
+      </c>
       <c r="B180" t="s">
         <v>184</v>
       </c>
@@ -4091,7 +4626,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="181" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>215</v>
+      </c>
       <c r="B181" t="s">
         <v>185</v>
       </c>
@@ -4108,7 +4646,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="182" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>215</v>
+      </c>
       <c r="B182" t="s">
         <v>186</v>
       </c>
@@ -4125,7 +4666,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="183" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>215</v>
+      </c>
       <c r="B183" t="s">
         <v>187</v>
       </c>
@@ -4142,7 +4686,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="184" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>215</v>
+      </c>
       <c r="B184" t="s">
         <v>188</v>
       </c>
@@ -4159,7 +4706,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="185" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>215</v>
+      </c>
       <c r="B185" t="s">
         <v>189</v>
       </c>
@@ -4176,7 +4726,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="186" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>215</v>
+      </c>
       <c r="B186" t="s">
         <v>190</v>
       </c>
@@ -4193,44 +4746,53 @@
         <v>8</v>
       </c>
     </row>
-    <row r="187" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>215</v>
+      </c>
       <c r="B187" t="s">
+        <v>154</v>
+      </c>
+      <c r="C187">
+        <v>0</v>
+      </c>
+      <c r="D187">
+        <v>0</v>
+      </c>
+      <c r="E187">
+        <v>0</v>
+      </c>
+      <c r="F187" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>215</v>
+      </c>
+      <c r="B188" t="s">
         <v>191</v>
       </c>
-      <c r="C187">
-        <v>0</v>
-      </c>
-      <c r="D187">
-        <v>0</v>
-      </c>
-      <c r="E187">
-        <v>0</v>
-      </c>
-      <c r="F187" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="188" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B188" t="s">
+      <c r="C188">
+        <v>0</v>
+      </c>
+      <c r="D188">
+        <v>0</v>
+      </c>
+      <c r="E188">
+        <v>0</v>
+      </c>
+      <c r="F188" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>215</v>
+      </c>
+      <c r="B189" t="s">
         <v>192</v>
       </c>
-      <c r="C188">
-        <v>0</v>
-      </c>
-      <c r="D188">
-        <v>0</v>
-      </c>
-      <c r="E188">
-        <v>0</v>
-      </c>
-      <c r="F188" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="189" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B189" t="s">
-        <v>154</v>
-      </c>
       <c r="C189">
         <v>0</v>
       </c>
@@ -4244,7 +4806,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="190" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>215</v>
+      </c>
       <c r="B190" t="s">
         <v>193</v>
       </c>
@@ -4261,7 +4826,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="191" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>215</v>
+      </c>
       <c r="B191" t="s">
         <v>194</v>
       </c>
@@ -4278,7 +4846,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="192" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>215</v>
+      </c>
       <c r="B192" t="s">
         <v>195</v>
       </c>
@@ -4295,7 +4866,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="193" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>215</v>
+      </c>
       <c r="B193" t="s">
         <v>196</v>
       </c>
@@ -4312,7 +4886,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="194" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>215</v>
+      </c>
       <c r="B194" t="s">
         <v>197</v>
       </c>
@@ -4329,7 +4906,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="195" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>215</v>
+      </c>
       <c r="B195" t="s">
         <v>198</v>
       </c>
@@ -4346,7 +4926,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="196" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>215</v>
+      </c>
       <c r="B196" t="s">
         <v>199</v>
       </c>
@@ -4363,7 +4946,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="197" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>215</v>
+      </c>
       <c r="B197" t="s">
         <v>200</v>
       </c>
@@ -4380,7 +4966,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="198" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>215</v>
+      </c>
       <c r="B198" t="s">
         <v>201</v>
       </c>
@@ -4397,7 +4986,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="199" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>215</v>
+      </c>
       <c r="B199" t="s">
         <v>202</v>
       </c>
@@ -4414,7 +5006,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="200" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>215</v>
+      </c>
       <c r="B200" t="s">
         <v>203</v>
       </c>
@@ -4431,7 +5026,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="201" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>215</v>
+      </c>
       <c r="B201" t="s">
         <v>204</v>
       </c>
@@ -4448,7 +5046,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="202" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>215</v>
+      </c>
       <c r="B202" t="s">
         <v>205</v>
       </c>
@@ -4465,7 +5066,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="203" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>217</v>
+      </c>
       <c r="B203" t="s">
         <v>206</v>
       </c>
@@ -4482,7 +5086,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="204" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>217</v>
+      </c>
       <c r="B204" t="s">
         <v>207</v>
       </c>
@@ -4499,7 +5106,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="205" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>217</v>
+      </c>
       <c r="B205" t="s">
         <v>208</v>
       </c>
@@ -4516,7 +5126,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="206" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>217</v>
+      </c>
       <c r="B206" t="s">
         <v>209</v>
       </c>
@@ -4533,7 +5146,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="207" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>217</v>
+      </c>
       <c r="B207" t="s">
         <v>210</v>
       </c>
@@ -4550,7 +5166,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="208" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>217</v>
+      </c>
       <c r="B208" t="s">
         <v>211</v>
       </c>
@@ -4567,7 +5186,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="209" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>217</v>
+      </c>
       <c r="B209" t="s">
         <v>212</v>
       </c>
@@ -4584,7 +5206,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="210" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>217</v>
+      </c>
       <c r="B210" t="s">
         <v>213</v>
       </c>
@@ -4598,40 +5223,6 @@
         <v>0</v>
       </c>
       <c r="F210" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="211" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B211" t="s">
-        <v>214</v>
-      </c>
-      <c r="C211">
-        <v>0</v>
-      </c>
-      <c r="D211">
-        <v>0</v>
-      </c>
-      <c r="E211">
-        <v>0</v>
-      </c>
-      <c r="F211" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="212" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B212" t="s">
-        <v>215</v>
-      </c>
-      <c r="C212">
-        <v>0</v>
-      </c>
-      <c r="D212">
-        <v>0</v>
-      </c>
-      <c r="E212">
-        <v>0</v>
-      </c>
-      <c r="F212" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>